<commit_message>
fix: Corrigi os pesos da Cota de Malha
</commit_message>
<xml_diff>
--- a/app/data/armors.xlsx
+++ b/app/data/armors.xlsx
@@ -1363,7 +1363,7 @@
         <v>5.0</v>
       </c>
       <c r="H22" s="11">
-        <v>10.0</v>
+        <v>8.0</v>
       </c>
       <c r="I22" s="3">
         <v>800.0</v>
@@ -1398,7 +1398,7 @@
         <v>7.0</v>
       </c>
       <c r="H23" s="11">
-        <v>9.8</v>
+        <v>8.9</v>
       </c>
       <c r="I23" s="3">
         <v>1600.0</v>
@@ -1433,7 +1433,7 @@
         <v>9.0</v>
       </c>
       <c r="H24" s="11">
-        <v>9.6</v>
+        <v>8.8</v>
       </c>
       <c r="I24" s="3">
         <v>3200.0</v>
@@ -1468,7 +1468,7 @@
         <v>11.0</v>
       </c>
       <c r="H25" s="11">
-        <v>9.4</v>
+        <v>8.7</v>
       </c>
       <c r="I25" s="3">
         <v>6400.0</v>
@@ -1503,7 +1503,7 @@
         <v>13.0</v>
       </c>
       <c r="H26" s="11">
-        <v>9.2</v>
+        <v>8.6</v>
       </c>
       <c r="I26" s="3">
         <v>12800.0</v>

</xml_diff>